<commit_message>
update general y datos
Cambiadas pestañas R delante
Subidos datasets actualizados
</commit_message>
<xml_diff>
--- a/datos/01-precio-leche.xlsx
+++ b/datos/01-precio-leche.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/34bf2af71bbc2e43/Documentos/GitHub/master-queseria/website/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="91" documentId="8_{C3D8DB6E-80F1-4A74-A94C-632DB8A5E2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93EED132-CBDA-4567-800A-682B281B9926}"/>
+  <xr:revisionPtr revIDLastSave="99" documentId="8_{C3D8DB6E-80F1-4A74-A94C-632DB8A5E2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22591ADE-EC19-467B-8AB7-BF1170373551}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="23595" windowHeight="14250" tabRatio="675" xr2:uid="{6977E7F1-D64B-47FE-B2A7-D4E9B0399E18}"/>
+    <workbookView xWindow="3165" yWindow="885" windowWidth="23595" windowHeight="14250" tabRatio="675" activeTab="1" xr2:uid="{6977E7F1-D64B-47FE-B2A7-D4E9B0399E18}"/>
   </bookViews>
   <sheets>
     <sheet name="Liquidación leche" sheetId="17" r:id="rId1"/>

</xml_diff>